<commit_message>
feat: publish priced five-board BOM and validated prototype manufacturing draft
</commit_message>
<xml_diff>
--- a/kicad-bare-nrf52840/procurement/digikey-2026-10-21/Plant-Monitor-BOM-DigiKey.xlsx
+++ b/kicad-bare-nrf52840/procurement/digikey-2026-10-21/Plant-Monitor-BOM-DigiKey.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM and cost" sheetId="1" r:id="R16f3f10b2dc84f84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM and cost" sheetId="1" r:id="Rcf66974e939c46e4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -45,7 +45,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -75,6 +75,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2EFDA"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -132,7 +137,7 @@
     <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -491,11 +496,11 @@
       </x:c>
       <x:c r="B5" s="3" t="n">
         <x:f>SUM(I11:I41)</x:f>
-        <x:v>90.58999999999999</x:v>
+        <x:v>90.69</x:v>
       </x:c>
       <x:c r="C5" s="1"/>
       <x:c r="D5" s="1" t="str">
-        <x:v>31 proposed lines in stock. AE1 is a conditional candidate requiring RF validation; C6 has reduced effective capacitance and requires supply-transient validation.</x:v>
+        <x:v>All 31 lines in stock. PCB updated for antenna A and 0603 C6. Antenna matching requires prototype RF validation.</x:v>
       </x:c>
       <x:c r="E5" s="1"/>
       <x:c r="F5" s="1"/>
@@ -515,8 +520,8 @@
         <x:v>Assembly release status</x:v>
       </x:c>
       <x:c r="B6" s="22" t="str">
-        <x:f>IF(T11="HOLD — RF validation","AE1/C6 HOLD","Review complete")</x:f>
-        <x:v>AE1/C6 HOLD</x:v>
+        <x:f>IF(T11="HOLD — RF validation","RF PROTOTYPE HOLD","Review complete")</x:f>
+        <x:v>RF PROTOTYPE HOLD</x:v>
       </x:c>
       <x:c r="C6" s="1"/>
       <x:c r="D6" s="1" t="str">
@@ -545,7 +550,7 @@
       </x:c>
       <x:c r="C7" s="1"/>
       <x:c r="D7" s="1" t="str">
-        <x:v>Procurement BOM only: CAD and submitted JLCPCB files unchanged. No purchase made. Requote if quantities change.</x:v>
+        <x:v>Schematic and PCB updated. Prior JLCPCB submission is stale; use revised draft files after review. No parts purchased.</x:v>
       </x:c>
       <x:c r="E7" s="1"/>
       <x:c r="F7" s="1"/>
@@ -566,11 +571,11 @@
       </x:c>
       <x:c r="B8" s="3" t="n">
         <x:f>B5-I11</x:f>
-        <x:v>87.99</x:v>
+        <x:v>88.09</x:v>
       </x:c>
       <x:c r="C8" s="1"/>
       <x:c r="D8" s="1" t="str">
-        <x:v>Antenna A candidate: $2.60 / five. Original B: $2.65 / five, out of stock; expected Nov 6. Neither option removes prototype RF qualification.</x:v>
+        <x:v>Antenna A: $2.60 / five. C19/L4/L5 = 1 pF / 2.7 nH / 3.9 nH prototype starting values; tune on assembled PCB.</x:v>
       </x:c>
       <x:c r="E8" s="1"/>
       <x:c r="F8" s="1"/>
@@ -709,7 +714,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="N11" s="9" t="str">
-        <x:v>Candidate only, NOT an approved drop-in. Same 3.2 x 1.6 mm body; 1=feed/2=NC; 2.4–2.5 GHz. PCB pads 1.2 x 1.8 mm at 2.9 mm pitch fit. A reference tuning is 1.0 pF / 2.7 nH / 3.9 nH; PCB has 1.2 pF / 2.7 nH / 3.3 nH. Requires board-specific matching, VNA and BLE-range validation. Original B antenna out of stock.</x:v>
+        <x:v>PCB updated for 2450AT18A0100001E: same 3.2 x 1.6 mm body and 1=feed/2=NC pads. Corrected all-copper corner clearance. C19/L4/L5 set to 1 pF / 2.7 nH / 3.9 nH as prototype starting values from manufacturer evaluation design. Board-specific VNA matching and BLE range validation required; not production-qualified.</x:v>
       </x:c>
       <x:c r="O11" s="9" t="str"/>
       <x:c r="P11" s="9" t="str">
@@ -999,10 +1004,10 @@
         <x:v>4.7u</x:v>
       </x:c>
       <x:c r="C16" s="9" t="str">
-        <x:v>C1005X5R1A475K050BC</x:v>
+        <x:v>GRM188R61C475KE11J</x:v>
       </x:c>
       <x:c r="D16" s="9" t="str">
-        <x:v>TDK</x:v>
+        <x:v>Murata</x:v>
       </x:c>
       <x:c r="E16" s="12" t="n">
         <x:v>1</x:v>
@@ -1012,33 +1017,33 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G16" s="9" t="str">
-        <x:v>445-13820-1-ND</x:v>
+        <x:v>490-GRM188R61C475KE11JCT-ND</x:v>
       </x:c>
       <x:c r="H16" s="10" t="n">
-        <x:v>0.25</x:v>
+        <x:v>0.26</x:v>
       </x:c>
       <x:c r="I16" s="11" t="n">
         <x:f>IF(ISNUMBER(H16),ROUND(F16*H16,2),"")</x:f>
-        <x:v>1.25</x:v>
+        <x:v>1.3</x:v>
       </x:c>
       <x:c r="J16" s="13" t="n">
-        <x:v>1492800</x:v>
+        <x:v>25063</x:v>
       </x:c>
       <x:c r="K16" s="9" t="str">
-        <x:v>In stock — review hold</x:v>
+        <x:v>In stock</x:v>
       </x:c>
       <x:c r="L16" s="9" t="str">
         <x:v>Cut Tape (CT) : 1</x:v>
       </x:c>
       <x:c r="M16" s="9" t="str">
-        <x:v>28</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="N16" s="9" t="str">
-        <x:v>Candidate only. 4.7 µF ±10% (was ±20%), 10 V X5R; 0402 body 1.0 x 0.5 mm, height ≤0.65 mm fits PCB pads. Typical manufacturer curves at 3 V: TDK about 1.4 µF, original Samsung about 1.8–1.9 µF (graph estimates, not guaranteed limits). Reduced effective bulk capacitance prevents unconditional equivalence approval. Verify VDD droop during worst-case BLE bursts with aged/cold CR2032 or select a characterized alternative.</x:v>
+        <x:v>4.7 µF ±10%, 16 V X5R. Changed PCB footprint to 0603 (1.6 x 0.8 mm), rotated and rerouted beside MCU; native DRC verifies clearances/connectivity. Manufacturer typical DC-bias curve indicates about 3.5 µF at 3 V, not a guaranteed minimum. J suffix is reel packaging. Verify battery supply droop during prototype BLE bursts.</x:v>
       </x:c>
       <x:c r="O16" s="9" t="str"/>
       <x:c r="P16" s="9" t="str">
-        <x:v>https://www.digikey.com/en/products/detail/tdk/C1005X5R1A475K050BC/3951056</x:v>
+        <x:v>https://www.digikey.com/en/products/detail/murata-electronics/GRM188R61C475KE11J/4905342</x:v>
       </x:c>
       <x:c r="Q16" s="9" t="str">
         <x:v>CL05A475MP5NRNC</x:v>
@@ -1047,13 +1052,13 @@
         <x:v>Samsung</x:v>
       </x:c>
       <x:c r="S16" s="9" t="str">
-        <x:v>Capacitor_SMD:C_0402_1005Metric</x:v>
+        <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
       </x:c>
       <x:c r="T16" s="21" t="str">
-        <x:v>HOLD — VDD transient validation</x:v>
+        <x:v>Reviewed — PCB footprint changed</x:v>
       </x:c>
       <x:c r="U16" s="9" t="str">
-        <x:v>https://product.tdk.com/system/files/dam/doc/product/capacitor/ceramic/mlcc/catalog/mlcc_commercial_general_en.pdf</x:v>
+        <x:v>https://mm.digikey.com/Volume0/opasdata/d220001/medias/docus/8942/490_Chip_Multilayer_CAT2021_MLCC.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="48" customHeight="1">
@@ -1451,10 +1456,10 @@
         <x:v>C19</x:v>
       </x:c>
       <x:c r="B23" s="9" t="str">
-        <x:v>1.2p</x:v>
+        <x:v>1p</x:v>
       </x:c>
       <x:c r="C23" s="9" t="str">
-        <x:v>GRM1555C1H1R2BA01D</x:v>
+        <x:v>GRM1555C1H1R0BA01D</x:v>
       </x:c>
       <x:c r="D23" s="9" t="str">
         <x:v>Murata</x:v>
@@ -1467,20 +1472,20 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G23" s="9" t="str">
-        <x:v>490-6209-1-ND</x:v>
+        <x:v>490-6206-1-ND</x:v>
       </x:c>
       <x:c r="H23" s="10" t="n">
-        <x:v>0.1</x:v>
+        <x:v>0.11</x:v>
       </x:c>
       <x:c r="I23" s="11" t="n">
         <x:f>IF(ISNUMBER(H23),ROUND(F23*H23,2),"")</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.55</x:v>
       </x:c>
       <x:c r="J23" s="13" t="n">
-        <x:v>168682</x:v>
+        <x:v>20971</x:v>
       </x:c>
       <x:c r="K23" s="9" t="str">
-        <x:v>In stock</x:v>
+        <x:v>In stock — review hold</x:v>
       </x:c>
       <x:c r="L23" s="9" t="str">
         <x:v>Cut Tape (CT) : 1</x:v>
@@ -1489,11 +1494,11 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="N23" s="9" t="str">
-        <x:v>Exact existing project part retained; no new substitution.</x:v>
+        <x:v>1.0 pF ±0.1 pF, 50 V C0G, same 0402 footprint. Changed from 1.2 pF to antenna A evaluation-board starting value; final value requires VNA tuning.</x:v>
       </x:c>
       <x:c r="O23" s="9" t="str"/>
       <x:c r="P23" s="9" t="str">
-        <x:v>https://www.digikey.com/en/products/detail/murata-electronics/GRM1555C1H1R2BA01D/3693934</x:v>
+        <x:v>https://www.digikey.com/en/products/detail/murata-electronics/GRM1555C1H1R0BA01D/3693930</x:v>
       </x:c>
       <x:c r="Q23" s="9" t="str">
         <x:v>GRM1555C1H1R2BA01D</x:v>
@@ -1505,7 +1510,7 @@
         <x:v>Capacitor_SMD:C_0402_1005Metric</x:v>
       </x:c>
       <x:c r="T23" s="9" t="str">
-        <x:v>Original part retained</x:v>
+        <x:v>RF prototype tuning value</x:v>
       </x:c>
       <x:c r="U23" s="9" t="str">
         <x:v>https://mm.digikey.com/Volume0/opasdata/d220001/medias/docus/8942/490_Chip_Multilayer_CAT2021_MLCC.pdf</x:v>
@@ -1906,10 +1911,10 @@
         <x:v>L5</x:v>
       </x:c>
       <x:c r="B30" s="9" t="str">
-        <x:v>3.3n</x:v>
+        <x:v>3.9n</x:v>
       </x:c>
       <x:c r="C30" s="9" t="str">
-        <x:v>LQG15HS3N3S02D</x:v>
+        <x:v>LQG15HS3N9S02D</x:v>
       </x:c>
       <x:c r="D30" s="9" t="str">
         <x:v>Murata</x:v>
@@ -1922,7 +1927,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G30" s="9" t="str">
-        <x:v>490-2616-1-ND</x:v>
+        <x:v>490-2617-1-ND</x:v>
       </x:c>
       <x:c r="H30" s="10" t="n">
         <x:v>0.1</x:v>
@@ -1932,10 +1937,10 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="J30" s="13" t="n">
-        <x:v>37534</x:v>
+        <x:v>15161</x:v>
       </x:c>
       <x:c r="K30" s="9" t="str">
-        <x:v>In stock</x:v>
+        <x:v>In stock — review hold</x:v>
       </x:c>
       <x:c r="L30" s="9" t="str">
         <x:v>Cut Tape (CT) : 1</x:v>
@@ -1944,11 +1949,11 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="N30" s="9" t="str">
-        <x:v>Exact existing project part retained; no new substitution.</x:v>
+        <x:v>3.9 nH ±0.3 nH, 0402, 750 mA, 140 mΩ maximum DCR, minimum self-resonance 6 GHz per Murata specification. Same LQG15HS footprint family. Changed from 3.3 nH to antenna A evaluation-board starting value; final value requires VNA tuning.</x:v>
       </x:c>
       <x:c r="O30" s="9" t="str"/>
       <x:c r="P30" s="9" t="str">
-        <x:v>https://www.digikey.com/en/products/detail/murata-electronics/LQG15HS3N3S02D/662865</x:v>
+        <x:v>https://www.digikey.com/en/products/detail/murata-electronics/LQG15HS3N9S02D/662866</x:v>
       </x:c>
       <x:c r="Q30" s="9" t="str">
         <x:v>LQG15HS3N3S02D</x:v>
@@ -1960,7 +1965,7 @@
         <x:v>Inductor_SMD:L_0402_1005Metric</x:v>
       </x:c>
       <x:c r="T30" s="9" t="str">
-        <x:v>Original part retained</x:v>
+        <x:v>RF prototype tuning value</x:v>
       </x:c>
       <x:c r="U30" s="9" t="str">
         <x:v>https://pim.murata.com/asset/pim4/inductor/JELF243B-0010_PDF_INDUCTOR</x:v>
@@ -2527,7 +2532,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="N39" s="9" t="str">
-        <x:v>SHTC3-TR-2.5KS is the tape-and-reel ordering code for the existing SHTC3. No sensor change.</x:v>
+        <x:v>Exact SHTC3 sensor; SHTC3-TR-2.5KS is Sensirion’s 2500-unit reel ordering code, available as cut tape from DigiKey. Same DFN 2 x 2 x 0.75 mm, pinout, I2C protocol and 1.62–3.6 V range. No hardware or firmware substitution.</x:v>
       </x:c>
       <x:c r="O39" s="9" t="str"/>
       <x:c r="P39" s="9" t="str">
@@ -2729,7 +2734,7 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" t="str">
-        <x:v>C6 hold: typical curves indicate ~1.4 µF at 3 V versus ~1.8–1.9 µF original. Confirm VDD droop with aged/cold battery during worst-case BLE bursts or select another capacitor.</x:v>
+        <x:v>C6: Murata 4.7 µF/16 V/X5R in 0603; typical DC-bias curve ~3.5 µF at 3 V (not guaranteed). Footprint and routing updated. Check supply transients on prototype.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>